<commit_message>
Revert "read in gdp data, create four variables and join to existing data"
</commit_message>
<xml_diff>
--- a/clean-data/output/citizenship-norm-indicator-tables.xlsx
+++ b/clean-data/output/citizenship-norm-indicator-tables.xlsx
@@ -437,7 +437,7 @@
         <v>1999</v>
       </c>
       <c r="C2">
-        <v>0.929</v>
+        <v>0.9290000000000001</v>
       </c>
       <c r="D2">
         <v>0.6870000000000001</v>
@@ -504,7 +504,7 @@
         <v>0.772</v>
       </c>
       <c r="J3">
-        <v>0.679</v>
+        <v>0.6790000000000001</v>
       </c>
       <c r="K3">
         <v>0.6870000000000001</v>
@@ -578,10 +578,10 @@
         <v>0.9340000000000001</v>
       </c>
       <c r="D5">
-        <v>0.8139999999999999</v>
+        <v>0.814</v>
       </c>
       <c r="E5">
-        <v>0.804</v>
+        <v>0.8040000000000001</v>
       </c>
       <c r="F5">
         <v>0.863</v>
@@ -593,7 +593,7 @@
         <v>0.846</v>
       </c>
       <c r="I5">
-        <v>0.5679999999999999</v>
+        <v>0.568</v>
       </c>
       <c r="J5">
         <v>0.879</v>
@@ -636,19 +636,19 @@
         <v>0.72</v>
       </c>
       <c r="H6">
-        <v>0.8149999999999999</v>
+        <v>0.815</v>
       </c>
       <c r="I6">
         <v>0.419</v>
       </c>
       <c r="J6">
-        <v>0.555</v>
+        <v>0.5550000000000001</v>
       </c>
       <c r="K6">
         <v>0.579</v>
       </c>
       <c r="L6">
-        <v>0.5639999999999999</v>
+        <v>0.564</v>
       </c>
       <c r="M6">
         <v>0.387</v>
@@ -673,13 +673,13 @@
         <v>0.823</v>
       </c>
       <c r="E7">
-        <v>0.677</v>
+        <v>0.6770000000000001</v>
       </c>
       <c r="F7">
-        <v>0.8159999999999999</v>
+        <v>0.816</v>
       </c>
       <c r="G7">
-        <v>0.8149999999999999</v>
+        <v>0.815</v>
       </c>
       <c r="H7">
         <v>0.707</v>
@@ -688,10 +688,10 @@
         <v>0.799</v>
       </c>
       <c r="J7">
-        <v>0.676</v>
+        <v>0.6760000000000001</v>
       </c>
       <c r="K7">
-        <v>0.676</v>
+        <v>0.6760000000000001</v>
       </c>
       <c r="L7">
         <v>0.709</v>
@@ -952,7 +952,7 @@
         <v>0.903</v>
       </c>
       <c r="F13">
-        <v>0.804</v>
+        <v>0.8040000000000001</v>
       </c>
       <c r="G13">
         <v>0.903</v>
@@ -967,7 +967,7 @@
         <v>0.849</v>
       </c>
       <c r="K13">
-        <v>0.677</v>
+        <v>0.6770000000000001</v>
       </c>
       <c r="L13">
         <v>0.661</v>
@@ -1038,16 +1038,16 @@
         <v>0.974</v>
       </c>
       <c r="D15">
-        <v>0.9409999999999999</v>
+        <v>0.941</v>
       </c>
       <c r="E15">
-        <v>0.9419999999999999</v>
+        <v>0.942</v>
       </c>
       <c r="F15">
         <v>0.837</v>
       </c>
       <c r="G15">
-        <v>0.9389999999999999</v>
+        <v>0.939</v>
       </c>
       <c r="H15">
         <v>0.879</v>
@@ -1084,7 +1084,7 @@
         <v>0.875</v>
       </c>
       <c r="D16">
-        <v>0.9409999999999999</v>
+        <v>0.941</v>
       </c>
       <c r="E16">
         <v>0.898</v>
@@ -1191,7 +1191,7 @@
         <v>0.914</v>
       </c>
       <c r="I18">
-        <v>0.926</v>
+        <v>0.9260000000000001</v>
       </c>
       <c r="J18">
         <v>0.909</v>
@@ -1231,7 +1231,7 @@
         <v>0.718</v>
       </c>
       <c r="G19">
-        <v>0.805</v>
+        <v>0.8050000000000001</v>
       </c>
       <c r="H19">
         <v>0.821</v>
@@ -1277,10 +1277,10 @@
         <v>0.772</v>
       </c>
       <c r="G20">
-        <v>0.8159999999999999</v>
+        <v>0.816</v>
       </c>
       <c r="H20">
-        <v>0.68</v>
+        <v>0.6800000000000001</v>
       </c>
       <c r="I20">
         <v>0.716</v>
@@ -1314,7 +1314,7 @@
         <v>0.922</v>
       </c>
       <c r="D21">
-        <v>0.8169999999999999</v>
+        <v>0.817</v>
       </c>
       <c r="E21">
         <v>0.767</v>
@@ -1449,13 +1449,13 @@
         <v>2009</v>
       </c>
       <c r="C24">
-        <v>0.9429999999999999</v>
+        <v>0.943</v>
       </c>
       <c r="D24">
         <v>0.6879999999999999</v>
       </c>
       <c r="E24">
-        <v>0.554</v>
+        <v>0.5540000000000001</v>
       </c>
       <c r="F24">
         <v>0.75</v>
@@ -1467,7 +1467,7 @@
         <v>0.791</v>
       </c>
       <c r="I24">
-        <v>0.677</v>
+        <v>0.6770000000000001</v>
       </c>
       <c r="J24">
         <v>0.883</v>
@@ -1633,7 +1633,7 @@
         <v>2016</v>
       </c>
       <c r="C28">
-        <v>0.9389999999999999</v>
+        <v>0.939</v>
       </c>
       <c r="D28">
         <v>0.919</v>
@@ -1651,7 +1651,7 @@
         <v>0.77</v>
       </c>
       <c r="I28">
-        <v>0.9429999999999999</v>
+        <v>0.943</v>
       </c>
       <c r="J28">
         <v>0.916</v>
@@ -1688,7 +1688,7 @@
         <v>0.785</v>
       </c>
       <c r="F29">
-        <v>0.927</v>
+        <v>0.9270000000000001</v>
       </c>
       <c r="G29">
         <v>0.763</v>
@@ -1746,7 +1746,7 @@
         <v>0.628</v>
       </c>
       <c r="J30">
-        <v>0.801</v>
+        <v>0.8010000000000001</v>
       </c>
       <c r="K30">
         <v>0.712</v>
@@ -1789,7 +1789,7 @@
         <v>0.761</v>
       </c>
       <c r="I31">
-        <v>0.6889999999999999</v>
+        <v>0.689</v>
       </c>
       <c r="J31">
         <v>0.787</v>
@@ -1829,7 +1829,7 @@
         <v>0.827</v>
       </c>
       <c r="G32">
-        <v>0.681</v>
+        <v>0.6810000000000001</v>
       </c>
       <c r="H32">
         <v>0.701</v>
@@ -1881,7 +1881,7 @@
         <v>0.669</v>
       </c>
       <c r="I33">
-        <v>0.805</v>
+        <v>0.8050000000000001</v>
       </c>
       <c r="J33">
         <v>0.731</v>
@@ -2108,7 +2108,7 @@
         <v>0.888</v>
       </c>
       <c r="H38">
-        <v>0.9429999999999999</v>
+        <v>0.943</v>
       </c>
       <c r="I38">
         <v>0.881</v>
@@ -2157,7 +2157,7 @@
         <v>0.747</v>
       </c>
       <c r="I39">
-        <v>0.8179999999999999</v>
+        <v>0.818</v>
       </c>
       <c r="J39">
         <v>0.718</v>
@@ -2169,7 +2169,7 @@
         <v>0.778</v>
       </c>
       <c r="M39">
-        <v>0.5679999999999999</v>
+        <v>0.568</v>
       </c>
       <c r="N39">
         <v>0.267</v>
@@ -2203,7 +2203,7 @@
         <v>0.922</v>
       </c>
       <c r="I40">
-        <v>0.926</v>
+        <v>0.9260000000000001</v>
       </c>
       <c r="J40">
         <v>0.9</v>
@@ -2234,7 +2234,7 @@
         <v>0.944</v>
       </c>
       <c r="D41">
-        <v>0.801</v>
+        <v>0.8010000000000001</v>
       </c>
       <c r="E41">
         <v>0.852</v>
@@ -2323,7 +2323,7 @@
         <v>2016</v>
       </c>
       <c r="C43">
-        <v>0.93</v>
+        <v>0.9300000000000001</v>
       </c>
       <c r="D43">
         <v>0.773</v>
@@ -2369,7 +2369,7 @@
         <v>2016</v>
       </c>
       <c r="C44">
-        <v>0.9419999999999999</v>
+        <v>0.942</v>
       </c>
       <c r="D44">
         <v>0.907</v>
@@ -2381,7 +2381,7 @@
         <v>0.953</v>
       </c>
       <c r="G44">
-        <v>0.927</v>
+        <v>0.9270000000000001</v>
       </c>
       <c r="H44">
         <v>0.9</v>
@@ -2430,7 +2430,7 @@
         <v>0.765</v>
       </c>
       <c r="H45">
-        <v>0.8149999999999999</v>
+        <v>0.815</v>
       </c>
       <c r="I45">
         <v>0.858</v>
@@ -2467,10 +2467,10 @@
         <v>0.857</v>
       </c>
       <c r="E46">
-        <v>0.931</v>
+        <v>0.9310000000000001</v>
       </c>
       <c r="F46">
-        <v>0.9389999999999999</v>
+        <v>0.939</v>
       </c>
       <c r="G46">
         <v>0.9360000000000001</v>
@@ -2488,13 +2488,13 @@
         <v>0.743</v>
       </c>
       <c r="L46">
-        <v>0.806</v>
+        <v>0.8060000000000001</v>
       </c>
       <c r="M46">
         <v>0.482</v>
       </c>
       <c r="N46">
-        <v>0.551</v>
+        <v>0.5510000000000001</v>
       </c>
     </row>
     <row r="47">
@@ -2663,7 +2663,7 @@
         <v>0.91</v>
       </c>
       <c r="I50">
-        <v>0.928</v>
+        <v>0.9280000000000001</v>
       </c>
       <c r="J50">
         <v>0.828</v>
@@ -2737,7 +2737,7 @@
         <v>2016</v>
       </c>
       <c r="C52">
-        <v>0.9389999999999999</v>
+        <v>0.939</v>
       </c>
       <c r="D52">
         <v>0.836</v>
@@ -2752,7 +2752,7 @@
         <v>0.898</v>
       </c>
       <c r="H52">
-        <v>0.926</v>
+        <v>0.9260000000000001</v>
       </c>
       <c r="I52">
         <v>0.821</v>
@@ -2789,7 +2789,7 @@
         <v>0.714</v>
       </c>
       <c r="E53">
-        <v>0.681</v>
+        <v>0.6810000000000001</v>
       </c>
       <c r="F53">
         <v>0.626</v>
@@ -2798,7 +2798,7 @@
         <v>0.652</v>
       </c>
       <c r="H53">
-        <v>0.6899999999999999</v>
+        <v>0.69</v>
       </c>
       <c r="I53">
         <v>0.754</v>
@@ -2829,7 +2829,7 @@
         <v>1999</v>
       </c>
       <c r="C54">
-        <v>0.928</v>
+        <v>0.9280000000000001</v>
       </c>
       <c r="D54">
         <v>0.903</v>
@@ -2847,7 +2847,7 @@
         <v>0.839</v>
       </c>
       <c r="I54">
-        <v>0.806</v>
+        <v>0.8060000000000001</v>
       </c>
       <c r="J54">
         <v>0.76</v>
@@ -2859,7 +2859,7 @@
         <v>0.721</v>
       </c>
       <c r="M54">
-        <v>0.5649999999999999</v>
+        <v>0.565</v>
       </c>
       <c r="N54">
         <v>0.387</v>
@@ -2881,7 +2881,7 @@
         <v>0.765</v>
       </c>
       <c r="E55">
-        <v>0.8149999999999999</v>
+        <v>0.815</v>
       </c>
       <c r="F55">
         <v>0.745</v>
@@ -2890,7 +2890,7 @@
         <v>0.771</v>
       </c>
       <c r="H55">
-        <v>0.806</v>
+        <v>0.8060000000000001</v>
       </c>
       <c r="I55">
         <v>0.891</v>
@@ -2921,7 +2921,7 @@
         <v>2016</v>
       </c>
       <c r="C56">
-        <v>0.931</v>
+        <v>0.9310000000000001</v>
       </c>
       <c r="D56">
         <v>0.754</v>
@@ -2976,7 +2976,7 @@
         <v>0.665</v>
       </c>
       <c r="F57">
-        <v>0.679</v>
+        <v>0.6790000000000001</v>
       </c>
       <c r="G57">
         <v>0.748</v>
@@ -3022,7 +3022,7 @@
         <v>0.726</v>
       </c>
       <c r="F58">
-        <v>0.801</v>
+        <v>0.8010000000000001</v>
       </c>
       <c r="G58">
         <v>0.761</v>
@@ -3123,10 +3123,10 @@
         <v>0.791</v>
       </c>
       <c r="I60">
-        <v>0.805</v>
+        <v>0.8050000000000001</v>
       </c>
       <c r="J60">
-        <v>0.8169999999999999</v>
+        <v>0.817</v>
       </c>
       <c r="K60">
         <v>0.785</v>
@@ -3169,7 +3169,7 @@
         <v>0.87</v>
       </c>
       <c r="I61">
-        <v>0.8159999999999999</v>
+        <v>0.816</v>
       </c>
       <c r="J61">
         <v>0.784</v>
@@ -3295,7 +3295,7 @@
         <v>0.849</v>
       </c>
       <c r="E64">
-        <v>0.803</v>
+        <v>0.8030000000000001</v>
       </c>
       <c r="F64">
         <v>0.834</v>
@@ -3356,7 +3356,7 @@
         <v>0.46</v>
       </c>
       <c r="J65">
-        <v>0.805</v>
+        <v>0.8050000000000001</v>
       </c>
       <c r="K65">
         <v>0.668</v>
@@ -3454,7 +3454,7 @@
         <v>0.671</v>
       </c>
       <c r="L67">
-        <v>0.676</v>
+        <v>0.6760000000000001</v>
       </c>
       <c r="M67">
         <v>0.362</v>
@@ -3497,7 +3497,7 @@
         <v>0.86</v>
       </c>
       <c r="K68">
-        <v>0.801</v>
+        <v>0.8010000000000001</v>
       </c>
       <c r="L68">
         <v>0.697</v>
@@ -3519,7 +3519,7 @@
         <v>2016</v>
       </c>
       <c r="C69">
-        <v>0.928</v>
+        <v>0.9280000000000001</v>
       </c>
       <c r="D69">
         <v>0.8110000000000001</v>
@@ -3589,7 +3589,7 @@
         <v>0.788</v>
       </c>
       <c r="K70">
-        <v>0.6919999999999999</v>
+        <v>0.692</v>
       </c>
       <c r="L70">
         <v>0.529</v>
@@ -3629,7 +3629,7 @@
         <v>0.951</v>
       </c>
       <c r="I71">
-        <v>0.9399999999999999</v>
+        <v>0.94</v>
       </c>
       <c r="J71">
         <v>0.92</v>
@@ -3660,7 +3660,7 @@
         <v>0.961</v>
       </c>
       <c r="D72">
-        <v>0.8169999999999999</v>
+        <v>0.817</v>
       </c>
       <c r="E72">
         <v>0.907</v>
@@ -3678,7 +3678,7 @@
         <v>0.898</v>
       </c>
       <c r="J72">
-        <v>0.8159999999999999</v>
+        <v>0.816</v>
       </c>
       <c r="K72">
         <v>0.861</v>
@@ -3687,7 +3687,7 @@
         <v>0.766</v>
       </c>
       <c r="M72">
-        <v>0.553</v>
+        <v>0.5530000000000001</v>
       </c>
       <c r="N72">
         <v>0.387</v>
@@ -3715,7 +3715,7 @@
         <v>0.641</v>
       </c>
       <c r="G73">
-        <v>0.8169999999999999</v>
+        <v>0.817</v>
       </c>
       <c r="H73">
         <v>0.891</v>
@@ -3755,10 +3755,10 @@
         <v>0.883</v>
       </c>
       <c r="E74">
-        <v>0.9399999999999999</v>
+        <v>0.94</v>
       </c>
       <c r="F74">
-        <v>0.8159999999999999</v>
+        <v>0.816</v>
       </c>
       <c r="G74">
         <v>0.921</v>
@@ -3773,7 +3773,7 @@
         <v>0.828</v>
       </c>
       <c r="K74">
-        <v>0.8149999999999999</v>
+        <v>0.815</v>
       </c>
       <c r="L74">
         <v>0.734</v>
@@ -3868,7 +3868,7 @@
         <v>0.782</v>
       </c>
       <c r="L76">
-        <v>0.68</v>
+        <v>0.6800000000000001</v>
       </c>
       <c r="M76">
         <v>0.5629999999999999</v>
@@ -3899,7 +3899,7 @@
         <v>0.887</v>
       </c>
       <c r="G77">
-        <v>0.802</v>
+        <v>0.8020000000000001</v>
       </c>
       <c r="H77">
         <v>0.791</v>
@@ -3939,7 +3939,7 @@
         <v>0.827</v>
       </c>
       <c r="E78">
-        <v>0.801</v>
+        <v>0.8010000000000001</v>
       </c>
       <c r="F78">
         <v>0.821</v>
@@ -3957,10 +3957,10 @@
         <v>0.849</v>
       </c>
       <c r="K78">
-        <v>0.805</v>
+        <v>0.8050000000000001</v>
       </c>
       <c r="L78">
-        <v>0.68</v>
+        <v>0.6800000000000001</v>
       </c>
       <c r="M78">
         <v>0.454</v>
@@ -3985,7 +3985,7 @@
         <v>0.8080000000000001</v>
       </c>
       <c r="E79">
-        <v>0.8139999999999999</v>
+        <v>0.814</v>
       </c>
       <c r="F79">
         <v>0.836</v>
@@ -4028,7 +4028,7 @@
         <v>0.985</v>
       </c>
       <c r="D80">
-        <v>0.931</v>
+        <v>0.9310000000000001</v>
       </c>
       <c r="E80">
         <v>0.872</v>
@@ -4095,7 +4095,7 @@
         <v>0.534</v>
       </c>
       <c r="K81">
-        <v>0.6929999999999999</v>
+        <v>0.693</v>
       </c>
       <c r="L81">
         <v>0.536</v>
@@ -4190,7 +4190,7 @@
         <v>0.57</v>
       </c>
       <c r="L83">
-        <v>0.556</v>
+        <v>0.5560000000000001</v>
       </c>
       <c r="M83">
         <v>0.344</v>
@@ -4396,13 +4396,13 @@
         <v>0.949</v>
       </c>
       <c r="D88">
-        <v>0.926</v>
+        <v>0.9260000000000001</v>
       </c>
       <c r="E88">
         <v>0.9330000000000001</v>
       </c>
       <c r="F88">
-        <v>0.5639999999999999</v>
+        <v>0.564</v>
       </c>
       <c r="G88">
         <v>0.949</v>
@@ -4411,7 +4411,7 @@
         <v>0.973</v>
       </c>
       <c r="I88">
-        <v>0.93</v>
+        <v>0.9300000000000001</v>
       </c>
       <c r="J88">
         <v>0.825</v>
@@ -4503,7 +4503,7 @@
         <v>0.779</v>
       </c>
       <c r="I90">
-        <v>0.8179999999999999</v>
+        <v>0.818</v>
       </c>
       <c r="J90">
         <v>0.772</v>
@@ -4512,7 +4512,7 @@
         <v>0.899</v>
       </c>
       <c r="L90">
-        <v>0.681</v>
+        <v>0.6810000000000001</v>
       </c>
       <c r="M90">
         <v>0.595</v>

</xml_diff>